<commit_message>
chore: publish ekg IG 2.0.0-trial-use-2026-04-28
</commit_message>
<xml_diff>
--- a/ig/ekg/StructureDefinition-medcom-ekg-recording-bundle.xlsx
+++ b/ig/ekg/StructureDefinition-medcom-ekg-recording-bundle.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.2</t>
+    <t>2.0.0-trial-use-2026-04-28</t>
   </si>
   <si>
     <t>Name</t>
@@ -48,7 +48,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>active</t>
+    <t>draft</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-01-28T10:08:45+00:00</t>
+    <t>2026-04-29T09:39:42+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
chore: publish ekg IG 2.0.0-trial-use-2026-04-28 (#76)
Co-authored-by: SGA-MedCom <SGA-MedCom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ig/ekg/StructureDefinition-medcom-ekg-recording-bundle.xlsx
+++ b/ig/ekg/StructureDefinition-medcom-ekg-recording-bundle.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.2</t>
+    <t>2.0.0-trial-use-2026-04-28</t>
   </si>
   <si>
     <t>Name</t>
@@ -48,7 +48,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>active</t>
+    <t>draft</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-01-28T10:08:45+00:00</t>
+    <t>2026-04-29T09:39:42+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
chore: publish ekg IG 2.0.0
</commit_message>
<xml_diff>
--- a/ig/ekg/StructureDefinition-medcom-ekg-recording-bundle.xlsx
+++ b/ig/ekg/StructureDefinition-medcom-ekg-recording-bundle.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0.0-trial-use-2026-04-28</t>
+    <t>2.0.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -48,7 +48,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>draft</t>
+    <t>active</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-29T09:39:42+00:00</t>
+    <t>2026-06-04T11:20:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
chore: publish ekg IG 2.0.0 (#83)
Co-authored-by: RikkeVestesen <RikkeVestesen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ig/ekg/StructureDefinition-medcom-ekg-recording-bundle.xlsx
+++ b/ig/ekg/StructureDefinition-medcom-ekg-recording-bundle.xlsx
@@ -33,7 +33,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0.0-trial-use-2026-04-28</t>
+    <t>2.0.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -48,7 +48,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>draft</t>
+    <t>active</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-29T09:39:42+00:00</t>
+    <t>2026-06-04T11:20:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>